<commit_message>
Organik bölümdeki formlar yeni tasarıma (yeşil bant, GOTS+EMS logo) getirildi
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6foNXTwf1dGzDjULYpfrk
</commit_message>
<xml_diff>
--- a/formlar/10. Depo ve Sevkiyat/EMS.DP.FRM.08.01. Mal Kabul Kayıt Formu.xlsx
+++ b/formlar/10. Depo ve Sevkiyat/EMS.DP.FRM.08.01. Mal Kabul Kayıt Formu.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Form" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +69,37 @@
       <color rgb="00000000"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="28"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -92,8 +121,18 @@
         <fgColor rgb="00F6F7F9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00006600"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF1DE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -115,11 +154,121 @@
         <color rgb="009AA3B2"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="009AA3B2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="009AA3B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="009AA3B2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="009AA3B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009AA3B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="009AA3B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="009AA3B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009AA3B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="009AA3B2"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="009AA3B2"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="009AA3B2"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="009AA3B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="009AA3B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="009AA3B2"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="009AA3B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <top style="medium"/>
+    </border>
+    <border>
+      <top style="medium"/>
+    </border>
+    <border>
+      <left style="medium"/>
+    </border>
+    <border/>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -153,6 +302,48 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -230,32 +421,67 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
-      <colOff>0</colOff>
+      <colOff>238124</colOff>
       <row>0</row>
-      <rowOff>0</rowOff>
+      <rowOff>198193</rowOff>
     </from>
-    <ext cx="971550" cy="762000"/>
+    <to>
+      <col>2</col>
+      <colOff>171449</colOff>
+      <row>3</row>
+      <rowOff>205802</rowOff>
+    </to>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
-  </oneCellAnchor>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>11</col>
+      <colOff>66676</colOff>
+      <row>0</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>12</col>
+      <colOff>609600</colOff>
+      <row>3</row>
+      <rowOff>283176</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
 </wsDr>
 </file>
 
@@ -570,315 +796,317 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="n"/>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="A1" s="13" t="n"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="15" t="n"/>
+      <c r="D1" s="16" t="inlineStr">
         <is>
           <t>GOODS RECEIVING RECORD
 سجل استلام البضائع</t>
         </is>
       </c>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="14" t="n"/>
+      <c r="L1" s="14" t="n"/>
+      <c r="M1" s="14" t="n"/>
+      <c r="N1" s="17" t="inlineStr">
         <is>
           <t>DATE / التاريخ</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="O1" s="18" t="n"/>
+      <c r="P1" s="19" t="inlineStr">
         <is>
           <t>….../….../.…</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="A2" s="20" t="n"/>
+      <c r="B2" s="21" t="n"/>
+      <c r="C2" s="21" t="n"/>
+      <c r="D2" s="21" t="n"/>
+      <c r="E2" s="21" t="n"/>
+      <c r="F2" s="21" t="n"/>
+      <c r="G2" s="21" t="n"/>
+      <c r="H2" s="21" t="n"/>
+      <c r="I2" s="21" t="n"/>
+      <c r="J2" s="21" t="n"/>
+      <c r="K2" s="21" t="n"/>
+      <c r="L2" s="21" t="n"/>
+      <c r="M2" s="21" t="n"/>
+      <c r="N2" s="17" t="inlineStr">
         <is>
           <t>FORM NUMBER / رقم النموذج</t>
         </is>
       </c>
-      <c r="O2" s="2" t="n"/>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="O2" s="18" t="n"/>
+      <c r="P2" s="22" t="inlineStr">
         <is>
           <t>EMS.DP.FRM.08.01</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="n"/>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="A3" s="20" t="n"/>
+      <c r="B3" s="21" t="n"/>
+      <c r="C3" s="21" t="n"/>
+      <c r="D3" s="21" t="n"/>
+      <c r="E3" s="21" t="n"/>
+      <c r="F3" s="21" t="n"/>
+      <c r="G3" s="21" t="n"/>
+      <c r="H3" s="21" t="n"/>
+      <c r="I3" s="21" t="n"/>
+      <c r="J3" s="21" t="n"/>
+      <c r="K3" s="21" t="n"/>
+      <c r="L3" s="21" t="n"/>
+      <c r="M3" s="21" t="n"/>
+      <c r="N3" s="17" t="inlineStr">
         <is>
           <t>REVISION / المراجعة</t>
         </is>
       </c>
-      <c r="O3" s="2" t="n"/>
-      <c r="P3" s="1" t="inlineStr">
+      <c r="O3" s="18" t="n"/>
+      <c r="P3" s="19" t="inlineStr">
         <is>
           <t>R00</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="n"/>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="A4" s="20" t="n"/>
+      <c r="B4" s="21" t="n"/>
+      <c r="C4" s="21" t="n"/>
+      <c r="D4" s="21" t="n"/>
+      <c r="E4" s="21" t="n"/>
+      <c r="F4" s="21" t="n"/>
+      <c r="G4" s="21" t="n"/>
+      <c r="H4" s="21" t="n"/>
+      <c r="I4" s="21" t="n"/>
+      <c r="J4" s="21" t="n"/>
+      <c r="K4" s="21" t="n"/>
+      <c r="L4" s="21" t="n"/>
+      <c r="M4" s="21" t="n"/>
+      <c r="N4" s="17" t="inlineStr">
         <is>
           <t>PUBLIC. DATE / تاريخ النشر</t>
         </is>
       </c>
-      <c r="O4" s="2" t="n"/>
-      <c r="P4" s="1" t="inlineStr">
+      <c r="O4" s="18" t="n"/>
+      <c r="P4" s="19" t="inlineStr">
         <is>
           <t>14.10.2026</t>
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>RECEIVING INFORMATION / معلومات الاستلام</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
-      <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="n"/>
-      <c r="O6" s="2" t="n"/>
-      <c r="P6" s="2" t="n"/>
+      <c r="B6" s="24" t="n"/>
+      <c r="C6" s="24" t="n"/>
+      <c r="D6" s="24" t="n"/>
+      <c r="E6" s="24" t="n"/>
+      <c r="F6" s="24" t="n"/>
+      <c r="G6" s="24" t="n"/>
+      <c r="H6" s="24" t="n"/>
+      <c r="I6" s="24" t="n"/>
+      <c r="J6" s="24" t="n"/>
+      <c r="K6" s="24" t="n"/>
+      <c r="L6" s="24" t="n"/>
+      <c r="M6" s="24" t="n"/>
+      <c r="N6" s="24" t="n"/>
+      <c r="O6" s="24" t="n"/>
+      <c r="P6" s="25" t="n"/>
     </row>
     <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Date / Time
 التاريخ / الوقت</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="B7" s="24" t="n"/>
+      <c r="C7" s="24" t="n"/>
+      <c r="D7" s="25" t="n"/>
+      <c r="E7" s="26" t="inlineStr">
         <is>
           <t>Supplier
 المورد</t>
         </is>
       </c>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="F7" s="24" t="n"/>
+      <c r="G7" s="24" t="n"/>
+      <c r="H7" s="25" t="n"/>
+      <c r="I7" s="26" t="inlineStr">
         <is>
           <t>Delivery Note No
 رقم إشعار التسليم</t>
         </is>
       </c>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="8" t="n"/>
-      <c r="L7" s="8" t="n"/>
-      <c r="M7" s="7" t="inlineStr">
+      <c r="J7" s="24" t="n"/>
+      <c r="K7" s="24" t="n"/>
+      <c r="L7" s="25" t="n"/>
+      <c r="M7" s="26" t="inlineStr">
         <is>
           <t>Purchase Order No
 رقم أمر الشراء</t>
         </is>
       </c>
-      <c r="N7" s="8" t="n"/>
-      <c r="O7" s="8" t="n"/>
-      <c r="P7" s="8" t="n"/>
+      <c r="N7" s="24" t="n"/>
+      <c r="O7" s="24" t="n"/>
+      <c r="P7" s="25" t="n"/>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="26" t="inlineStr">
         <is>
           <t>Vehicle Plate / Driver
 لوحة المركبة / السائق</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="8" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="B8" s="24" t="n"/>
+      <c r="C8" s="24" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="26" t="inlineStr">
         <is>
           <t>Material Type
 نوع المادة (yarn / fabric / chemical / accessory / packaging)</t>
         </is>
       </c>
-      <c r="F8" s="8" t="n"/>
-      <c r="G8" s="8" t="n"/>
-      <c r="H8" s="8" t="n"/>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="F8" s="24" t="n"/>
+      <c r="G8" s="24" t="n"/>
+      <c r="H8" s="25" t="n"/>
+      <c r="I8" s="26" t="inlineStr">
         <is>
           <t>Warehouse Location
 موقع المستودع</t>
         </is>
       </c>
-      <c r="J8" s="8" t="n"/>
-      <c r="K8" s="8" t="n"/>
-      <c r="L8" s="8" t="n"/>
-      <c r="M8" s="7" t="inlineStr">
+      <c r="J8" s="24" t="n"/>
+      <c r="K8" s="24" t="n"/>
+      <c r="L8" s="25" t="n"/>
+      <c r="M8" s="26" t="inlineStr">
         <is>
           <t>Received By
 المستلم</t>
         </is>
       </c>
-      <c r="N8" s="8" t="n"/>
-      <c r="O8" s="8" t="n"/>
-      <c r="P8" s="8" t="n"/>
-    </row>
+      <c r="N8" s="24" t="n"/>
+      <c r="O8" s="24" t="n"/>
+      <c r="P8" s="25" t="n"/>
+    </row>
+    <row r="9"/>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>RECEIVED ITEMS / البنود المستلمة</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="n"/>
-      <c r="O10" s="2" t="n"/>
-      <c r="P10" s="2" t="n"/>
+      <c r="B10" s="24" t="n"/>
+      <c r="C10" s="24" t="n"/>
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="24" t="n"/>
+      <c r="F10" s="24" t="n"/>
+      <c r="G10" s="24" t="n"/>
+      <c r="H10" s="24" t="n"/>
+      <c r="I10" s="24" t="n"/>
+      <c r="J10" s="24" t="n"/>
+      <c r="K10" s="24" t="n"/>
+      <c r="L10" s="24" t="n"/>
+      <c r="M10" s="24" t="n"/>
+      <c r="N10" s="24" t="n"/>
+      <c r="O10" s="24" t="n"/>
+      <c r="P10" s="25" t="n"/>
     </row>
     <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>Item / Description
 الصنف / الوصف</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="C11" s="24" t="n"/>
+      <c r="D11" s="25" t="n"/>
+      <c r="E11" s="27" t="inlineStr">
         <is>
           <t>Lot / Batch No
 رقم الدفعة</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="F11" s="25" t="n"/>
+      <c r="G11" s="27" t="inlineStr">
         <is>
           <t>Ordered Qty
 المطلوب</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr">
+      <c r="H11" s="27" t="inlineStr">
         <is>
           <t>Delivery Note Qty
 حسب الإشعار</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr">
+      <c r="I11" s="27" t="inlineStr">
         <is>
           <t>Received Qty
 المستلم</t>
         </is>
       </c>
-      <c r="J11" s="9" t="inlineStr">
+      <c r="J11" s="27" t="inlineStr">
         <is>
           <t>Unit
 الوحدة</t>
         </is>
       </c>
-      <c r="K11" s="9" t="inlineStr">
+      <c r="K11" s="27" t="inlineStr">
         <is>
           <t>Packaging OK
 التغليف سليم</t>
         </is>
       </c>
-      <c r="L11" s="9" t="inlineStr">
+      <c r="L11" s="27" t="inlineStr">
         <is>
           <t>Label OK
 الملصق سليم</t>
         </is>
       </c>
-      <c r="M11" s="9" t="inlineStr">
+      <c r="M11" s="27" t="inlineStr">
         <is>
           <t>Result
 النتيجة (A/R/H)</t>
         </is>
       </c>
-      <c r="N11" s="9" t="inlineStr">
+      <c r="N11" s="27" t="inlineStr">
         <is>
           <t>Remarks
 ملاحظات</t>
         </is>
       </c>
-      <c r="O11" s="2" t="n"/>
-      <c r="P11" s="2" t="n"/>
+      <c r="O11" s="24" t="n"/>
+      <c r="P11" s="25" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="10" t="n">
         <v>1</v>
       </c>
       <c r="B12" s="10" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
+      <c r="C12" s="24" t="n"/>
+      <c r="D12" s="25" t="n"/>
       <c r="E12" s="10" t="n"/>
-      <c r="F12" s="2" t="n"/>
+      <c r="F12" s="25" t="n"/>
       <c r="G12" s="10" t="n"/>
       <c r="H12" s="10" t="n"/>
       <c r="I12" s="10" t="n"/>
@@ -887,18 +1115,18 @@
       <c r="L12" s="10" t="n"/>
       <c r="M12" s="10" t="n"/>
       <c r="N12" s="10" t="n"/>
-      <c r="O12" s="2" t="n"/>
-      <c r="P12" s="2" t="n"/>
+      <c r="O12" s="24" t="n"/>
+      <c r="P12" s="25" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="10" t="n">
         <v>2</v>
       </c>
       <c r="B13" s="10" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
+      <c r="C13" s="24" t="n"/>
+      <c r="D13" s="25" t="n"/>
       <c r="E13" s="10" t="n"/>
-      <c r="F13" s="2" t="n"/>
+      <c r="F13" s="25" t="n"/>
       <c r="G13" s="10" t="n"/>
       <c r="H13" s="10" t="n"/>
       <c r="I13" s="10" t="n"/>
@@ -907,18 +1135,18 @@
       <c r="L13" s="10" t="n"/>
       <c r="M13" s="10" t="n"/>
       <c r="N13" s="10" t="n"/>
-      <c r="O13" s="2" t="n"/>
-      <c r="P13" s="2" t="n"/>
+      <c r="O13" s="24" t="n"/>
+      <c r="P13" s="25" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="10" t="n">
         <v>3</v>
       </c>
       <c r="B14" s="10" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
+      <c r="C14" s="24" t="n"/>
+      <c r="D14" s="25" t="n"/>
       <c r="E14" s="10" t="n"/>
-      <c r="F14" s="2" t="n"/>
+      <c r="F14" s="25" t="n"/>
       <c r="G14" s="10" t="n"/>
       <c r="H14" s="10" t="n"/>
       <c r="I14" s="10" t="n"/>
@@ -927,18 +1155,18 @@
       <c r="L14" s="10" t="n"/>
       <c r="M14" s="10" t="n"/>
       <c r="N14" s="10" t="n"/>
-      <c r="O14" s="2" t="n"/>
-      <c r="P14" s="2" t="n"/>
+      <c r="O14" s="24" t="n"/>
+      <c r="P14" s="25" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="10" t="n">
         <v>4</v>
       </c>
       <c r="B15" s="10" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
+      <c r="C15" s="24" t="n"/>
+      <c r="D15" s="25" t="n"/>
       <c r="E15" s="10" t="n"/>
-      <c r="F15" s="2" t="n"/>
+      <c r="F15" s="25" t="n"/>
       <c r="G15" s="10" t="n"/>
       <c r="H15" s="10" t="n"/>
       <c r="I15" s="10" t="n"/>
@@ -947,18 +1175,18 @@
       <c r="L15" s="10" t="n"/>
       <c r="M15" s="10" t="n"/>
       <c r="N15" s="10" t="n"/>
-      <c r="O15" s="2" t="n"/>
-      <c r="P15" s="2" t="n"/>
+      <c r="O15" s="24" t="n"/>
+      <c r="P15" s="25" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="10" t="n">
         <v>5</v>
       </c>
       <c r="B16" s="10" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
+      <c r="C16" s="24" t="n"/>
+      <c r="D16" s="25" t="n"/>
       <c r="E16" s="10" t="n"/>
-      <c r="F16" s="2" t="n"/>
+      <c r="F16" s="25" t="n"/>
       <c r="G16" s="10" t="n"/>
       <c r="H16" s="10" t="n"/>
       <c r="I16" s="10" t="n"/>
@@ -967,18 +1195,18 @@
       <c r="L16" s="10" t="n"/>
       <c r="M16" s="10" t="n"/>
       <c r="N16" s="10" t="n"/>
-      <c r="O16" s="2" t="n"/>
-      <c r="P16" s="2" t="n"/>
+      <c r="O16" s="24" t="n"/>
+      <c r="P16" s="25" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="10" t="n">
         <v>6</v>
       </c>
       <c r="B17" s="10" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
+      <c r="C17" s="24" t="n"/>
+      <c r="D17" s="25" t="n"/>
       <c r="E17" s="10" t="n"/>
-      <c r="F17" s="2" t="n"/>
+      <c r="F17" s="25" t="n"/>
       <c r="G17" s="10" t="n"/>
       <c r="H17" s="10" t="n"/>
       <c r="I17" s="10" t="n"/>
@@ -987,18 +1215,18 @@
       <c r="L17" s="10" t="n"/>
       <c r="M17" s="10" t="n"/>
       <c r="N17" s="10" t="n"/>
-      <c r="O17" s="2" t="n"/>
-      <c r="P17" s="2" t="n"/>
+      <c r="O17" s="24" t="n"/>
+      <c r="P17" s="25" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="10" t="n">
         <v>7</v>
       </c>
       <c r="B18" s="10" t="n"/>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
+      <c r="C18" s="24" t="n"/>
+      <c r="D18" s="25" t="n"/>
       <c r="E18" s="10" t="n"/>
-      <c r="F18" s="2" t="n"/>
+      <c r="F18" s="25" t="n"/>
       <c r="G18" s="10" t="n"/>
       <c r="H18" s="10" t="n"/>
       <c r="I18" s="10" t="n"/>
@@ -1007,18 +1235,18 @@
       <c r="L18" s="10" t="n"/>
       <c r="M18" s="10" t="n"/>
       <c r="N18" s="10" t="n"/>
-      <c r="O18" s="2" t="n"/>
-      <c r="P18" s="2" t="n"/>
+      <c r="O18" s="24" t="n"/>
+      <c r="P18" s="25" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="10" t="n">
         <v>8</v>
       </c>
       <c r="B19" s="10" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="25" t="n"/>
       <c r="E19" s="10" t="n"/>
-      <c r="F19" s="2" t="n"/>
+      <c r="F19" s="25" t="n"/>
       <c r="G19" s="10" t="n"/>
       <c r="H19" s="10" t="n"/>
       <c r="I19" s="10" t="n"/>
@@ -1027,18 +1255,18 @@
       <c r="L19" s="10" t="n"/>
       <c r="M19" s="10" t="n"/>
       <c r="N19" s="10" t="n"/>
-      <c r="O19" s="2" t="n"/>
-      <c r="P19" s="2" t="n"/>
+      <c r="O19" s="24" t="n"/>
+      <c r="P19" s="25" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="10" t="n">
         <v>9</v>
       </c>
       <c r="B20" s="10" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
+      <c r="C20" s="24" t="n"/>
+      <c r="D20" s="25" t="n"/>
       <c r="E20" s="10" t="n"/>
-      <c r="F20" s="2" t="n"/>
+      <c r="F20" s="25" t="n"/>
       <c r="G20" s="10" t="n"/>
       <c r="H20" s="10" t="n"/>
       <c r="I20" s="10" t="n"/>
@@ -1047,18 +1275,18 @@
       <c r="L20" s="10" t="n"/>
       <c r="M20" s="10" t="n"/>
       <c r="N20" s="10" t="n"/>
-      <c r="O20" s="2" t="n"/>
-      <c r="P20" s="2" t="n"/>
+      <c r="O20" s="24" t="n"/>
+      <c r="P20" s="25" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="10" t="n">
         <v>10</v>
       </c>
       <c r="B21" s="10" t="n"/>
-      <c r="C21" s="2" t="n"/>
-      <c r="D21" s="2" t="n"/>
+      <c r="C21" s="24" t="n"/>
+      <c r="D21" s="25" t="n"/>
       <c r="E21" s="10" t="n"/>
-      <c r="F21" s="2" t="n"/>
+      <c r="F21" s="25" t="n"/>
       <c r="G21" s="10" t="n"/>
       <c r="H21" s="10" t="n"/>
       <c r="I21" s="10" t="n"/>
@@ -1067,18 +1295,18 @@
       <c r="L21" s="10" t="n"/>
       <c r="M21" s="10" t="n"/>
       <c r="N21" s="10" t="n"/>
-      <c r="O21" s="2" t="n"/>
-      <c r="P21" s="2" t="n"/>
+      <c r="O21" s="24" t="n"/>
+      <c r="P21" s="25" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="10" t="n">
         <v>11</v>
       </c>
       <c r="B22" s="10" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
+      <c r="C22" s="24" t="n"/>
+      <c r="D22" s="25" t="n"/>
       <c r="E22" s="10" t="n"/>
-      <c r="F22" s="2" t="n"/>
+      <c r="F22" s="25" t="n"/>
       <c r="G22" s="10" t="n"/>
       <c r="H22" s="10" t="n"/>
       <c r="I22" s="10" t="n"/>
@@ -1087,18 +1315,18 @@
       <c r="L22" s="10" t="n"/>
       <c r="M22" s="10" t="n"/>
       <c r="N22" s="10" t="n"/>
-      <c r="O22" s="2" t="n"/>
-      <c r="P22" s="2" t="n"/>
+      <c r="O22" s="24" t="n"/>
+      <c r="P22" s="25" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="10" t="n">
         <v>12</v>
       </c>
       <c r="B23" s="10" t="n"/>
-      <c r="C23" s="2" t="n"/>
-      <c r="D23" s="2" t="n"/>
+      <c r="C23" s="24" t="n"/>
+      <c r="D23" s="25" t="n"/>
       <c r="E23" s="10" t="n"/>
-      <c r="F23" s="2" t="n"/>
+      <c r="F23" s="25" t="n"/>
       <c r="G23" s="10" t="n"/>
       <c r="H23" s="10" t="n"/>
       <c r="I23" s="10" t="n"/>
@@ -1107,30 +1335,31 @@
       <c r="L23" s="10" t="n"/>
       <c r="M23" s="10" t="n"/>
       <c r="N23" s="10" t="n"/>
-      <c r="O23" s="2" t="n"/>
-      <c r="P23" s="2" t="n"/>
-    </row>
+      <c r="O23" s="24" t="n"/>
+      <c r="P23" s="25" t="n"/>
+    </row>
+    <row r="24"/>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="23" t="inlineStr">
         <is>
           <t>CHECKS / الفحوصات</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
-      <c r="J25" s="2" t="n"/>
-      <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="n"/>
-      <c r="M25" s="2" t="n"/>
-      <c r="N25" s="2" t="n"/>
-      <c r="O25" s="2" t="n"/>
-      <c r="P25" s="2" t="n"/>
+      <c r="B25" s="24" t="n"/>
+      <c r="C25" s="24" t="n"/>
+      <c r="D25" s="24" t="n"/>
+      <c r="E25" s="24" t="n"/>
+      <c r="F25" s="24" t="n"/>
+      <c r="G25" s="24" t="n"/>
+      <c r="H25" s="24" t="n"/>
+      <c r="I25" s="24" t="n"/>
+      <c r="J25" s="24" t="n"/>
+      <c r="K25" s="24" t="n"/>
+      <c r="L25" s="24" t="n"/>
+      <c r="M25" s="24" t="n"/>
+      <c r="N25" s="24" t="n"/>
+      <c r="O25" s="24" t="n"/>
+      <c r="P25" s="25" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
@@ -1138,43 +1367,44 @@
           <t>☐ Delivery note matches order / الإشعار مطابق للطلب   ☐ Quantity and lot match / الكمية والدفعة مطابقة   ☐ Packaging undamaged / التغليف غير تالف   ☐ Labels readable / الملصقات واضحة   ☐ Certificates and MSDS received / الشهادات ونشرة السلامة   ☐ Sent to quality inspection / أرسل لفحص الجودة</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="n"/>
-      <c r="J26" s="2" t="n"/>
-      <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
-      <c r="M26" s="2" t="n"/>
-      <c r="N26" s="2" t="n"/>
-      <c r="O26" s="2" t="n"/>
-      <c r="P26" s="2" t="n"/>
-    </row>
+      <c r="B26" s="24" t="n"/>
+      <c r="C26" s="24" t="n"/>
+      <c r="D26" s="24" t="n"/>
+      <c r="E26" s="24" t="n"/>
+      <c r="F26" s="24" t="n"/>
+      <c r="G26" s="24" t="n"/>
+      <c r="H26" s="24" t="n"/>
+      <c r="I26" s="24" t="n"/>
+      <c r="J26" s="24" t="n"/>
+      <c r="K26" s="24" t="n"/>
+      <c r="L26" s="24" t="n"/>
+      <c r="M26" s="24" t="n"/>
+      <c r="N26" s="24" t="n"/>
+      <c r="O26" s="24" t="n"/>
+      <c r="P26" s="25" t="n"/>
+    </row>
+    <row r="27"/>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="23" t="inlineStr">
         <is>
           <t>DECISION / القرار</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="n"/>
-      <c r="H28" s="2" t="n"/>
-      <c r="I28" s="2" t="n"/>
-      <c r="J28" s="2" t="n"/>
-      <c r="K28" s="2" t="n"/>
-      <c r="L28" s="2" t="n"/>
-      <c r="M28" s="2" t="n"/>
-      <c r="N28" s="2" t="n"/>
-      <c r="O28" s="2" t="n"/>
-      <c r="P28" s="2" t="n"/>
+      <c r="B28" s="24" t="n"/>
+      <c r="C28" s="24" t="n"/>
+      <c r="D28" s="24" t="n"/>
+      <c r="E28" s="24" t="n"/>
+      <c r="F28" s="24" t="n"/>
+      <c r="G28" s="24" t="n"/>
+      <c r="H28" s="24" t="n"/>
+      <c r="I28" s="24" t="n"/>
+      <c r="J28" s="24" t="n"/>
+      <c r="K28" s="24" t="n"/>
+      <c r="L28" s="24" t="n"/>
+      <c r="M28" s="24" t="n"/>
+      <c r="N28" s="24" t="n"/>
+      <c r="O28" s="24" t="n"/>
+      <c r="P28" s="25" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
@@ -1182,43 +1412,44 @@
           <t>☐ Accepted - stored / مقبول - مخزن   ☐ Hold - awaiting inspection / معلق بانتظار الفحص   ☐ Rejected - Non-conforming Material Notice / مرفوض</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="n"/>
-      <c r="H29" s="2" t="n"/>
-      <c r="I29" s="2" t="n"/>
-      <c r="J29" s="2" t="n"/>
-      <c r="K29" s="2" t="n"/>
-      <c r="L29" s="2" t="n"/>
-      <c r="M29" s="2" t="n"/>
-      <c r="N29" s="2" t="n"/>
-      <c r="O29" s="2" t="n"/>
-      <c r="P29" s="2" t="n"/>
-    </row>
+      <c r="B29" s="24" t="n"/>
+      <c r="C29" s="24" t="n"/>
+      <c r="D29" s="24" t="n"/>
+      <c r="E29" s="24" t="n"/>
+      <c r="F29" s="24" t="n"/>
+      <c r="G29" s="24" t="n"/>
+      <c r="H29" s="24" t="n"/>
+      <c r="I29" s="24" t="n"/>
+      <c r="J29" s="24" t="n"/>
+      <c r="K29" s="24" t="n"/>
+      <c r="L29" s="24" t="n"/>
+      <c r="M29" s="24" t="n"/>
+      <c r="N29" s="24" t="n"/>
+      <c r="O29" s="24" t="n"/>
+      <c r="P29" s="25" t="n"/>
+    </row>
+    <row r="30"/>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t>NOTES / ملاحظات</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="n"/>
-      <c r="J31" s="2" t="n"/>
-      <c r="K31" s="2" t="n"/>
-      <c r="L31" s="2" t="n"/>
-      <c r="M31" s="2" t="n"/>
-      <c r="N31" s="2" t="n"/>
-      <c r="O31" s="2" t="n"/>
-      <c r="P31" s="2" t="n"/>
+      <c r="B31" s="24" t="n"/>
+      <c r="C31" s="24" t="n"/>
+      <c r="D31" s="24" t="n"/>
+      <c r="E31" s="24" t="n"/>
+      <c r="F31" s="24" t="n"/>
+      <c r="G31" s="24" t="n"/>
+      <c r="H31" s="24" t="n"/>
+      <c r="I31" s="24" t="n"/>
+      <c r="J31" s="24" t="n"/>
+      <c r="K31" s="24" t="n"/>
+      <c r="L31" s="24" t="n"/>
+      <c r="M31" s="24" t="n"/>
+      <c r="N31" s="24" t="n"/>
+      <c r="O31" s="24" t="n"/>
+      <c r="P31" s="25" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
@@ -1226,148 +1457,139 @@
           <t>Shortages, damage, discrepancies and photo references.</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
-      <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="n"/>
-      <c r="J32" s="2" t="n"/>
-      <c r="K32" s="2" t="n"/>
-      <c r="L32" s="2" t="n"/>
-      <c r="M32" s="2" t="n"/>
-      <c r="N32" s="2" t="n"/>
-      <c r="O32" s="2" t="n"/>
-      <c r="P32" s="2" t="n"/>
+      <c r="B32" s="28" t="n"/>
+      <c r="C32" s="28" t="n"/>
+      <c r="D32" s="28" t="n"/>
+      <c r="E32" s="28" t="n"/>
+      <c r="F32" s="28" t="n"/>
+      <c r="G32" s="28" t="n"/>
+      <c r="H32" s="28" t="n"/>
+      <c r="I32" s="28" t="n"/>
+      <c r="J32" s="28" t="n"/>
+      <c r="K32" s="28" t="n"/>
+      <c r="L32" s="28" t="n"/>
+      <c r="M32" s="28" t="n"/>
+      <c r="N32" s="28" t="n"/>
+      <c r="O32" s="28" t="n"/>
+      <c r="P32" s="29" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
-      <c r="G33" s="2" t="n"/>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n"/>
-      <c r="J33" s="2" t="n"/>
-      <c r="K33" s="2" t="n"/>
-      <c r="L33" s="2" t="n"/>
-      <c r="M33" s="2" t="n"/>
-      <c r="N33" s="2" t="n"/>
-      <c r="O33" s="2" t="n"/>
-      <c r="P33" s="2" t="n"/>
-    </row>
+      <c r="A33" s="30" t="n"/>
+      <c r="B33" s="31" t="n"/>
+      <c r="C33" s="31" t="n"/>
+      <c r="D33" s="31" t="n"/>
+      <c r="E33" s="31" t="n"/>
+      <c r="F33" s="31" t="n"/>
+      <c r="G33" s="31" t="n"/>
+      <c r="H33" s="31" t="n"/>
+      <c r="I33" s="31" t="n"/>
+      <c r="J33" s="31" t="n"/>
+      <c r="K33" s="31" t="n"/>
+      <c r="L33" s="31" t="n"/>
+      <c r="M33" s="31" t="n"/>
+      <c r="N33" s="31" t="n"/>
+      <c r="O33" s="31" t="n"/>
+      <c r="P33" s="32" t="n"/>
+    </row>
+    <row r="34"/>
     <row r="35">
-      <c r="A35" s="9" t="inlineStr">
+      <c r="A35" s="27" t="inlineStr">
         <is>
           <t>Warehouse / المستودع</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="9" t="inlineStr">
+      <c r="B35" s="24" t="n"/>
+      <c r="C35" s="24" t="n"/>
+      <c r="D35" s="24" t="n"/>
+      <c r="E35" s="25" t="n"/>
+      <c r="F35" s="27" t="inlineStr">
         <is>
           <t>Quality / الجودة</t>
         </is>
       </c>
-      <c r="G35" s="2" t="n"/>
-      <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="n"/>
-      <c r="J35" s="2" t="n"/>
-      <c r="K35" s="9" t="inlineStr">
+      <c r="G35" s="24" t="n"/>
+      <c r="H35" s="24" t="n"/>
+      <c r="I35" s="24" t="n"/>
+      <c r="J35" s="25" t="n"/>
+      <c r="K35" s="27" t="inlineStr">
         <is>
           <t>Purchasing / المشتريات</t>
         </is>
       </c>
-      <c r="L35" s="2" t="n"/>
-      <c r="M35" s="2" t="n"/>
-      <c r="N35" s="2" t="n"/>
-      <c r="O35" s="2" t="n"/>
-      <c r="P35" s="2" t="n"/>
+      <c r="L35" s="24" t="n"/>
+      <c r="M35" s="24" t="n"/>
+      <c r="N35" s="24" t="n"/>
+      <c r="O35" s="24" t="n"/>
+      <c r="P35" s="25" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
+      <c r="B36" s="28" t="n"/>
+      <c r="C36" s="28" t="n"/>
+      <c r="D36" s="28" t="n"/>
+      <c r="E36" s="29" t="n"/>
       <c r="F36" s="1" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
-      <c r="J36" s="2" t="n"/>
+      <c r="G36" s="28" t="n"/>
+      <c r="H36" s="28" t="n"/>
+      <c r="I36" s="28" t="n"/>
+      <c r="J36" s="29" t="n"/>
       <c r="K36" s="1" t="n"/>
-      <c r="L36" s="2" t="n"/>
-      <c r="M36" s="2" t="n"/>
-      <c r="N36" s="2" t="n"/>
-      <c r="O36" s="2" t="n"/>
-      <c r="P36" s="2" t="n"/>
+      <c r="L36" s="28" t="n"/>
+      <c r="M36" s="28" t="n"/>
+      <c r="N36" s="28" t="n"/>
+      <c r="O36" s="28" t="n"/>
+      <c r="P36" s="29" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n"/>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
-      <c r="J37" s="2" t="n"/>
-      <c r="K37" s="2" t="n"/>
-      <c r="L37" s="2" t="n"/>
-      <c r="M37" s="2" t="n"/>
-      <c r="N37" s="2" t="n"/>
-      <c r="O37" s="2" t="n"/>
-      <c r="P37" s="2" t="n"/>
+      <c r="A37" s="33" t="n"/>
+      <c r="E37" s="34" t="n"/>
+      <c r="F37" s="33" t="n"/>
+      <c r="J37" s="34" t="n"/>
+      <c r="K37" s="33" t="n"/>
+      <c r="P37" s="34" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
-      <c r="G38" s="2" t="n"/>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="n"/>
-      <c r="J38" s="2" t="n"/>
-      <c r="K38" s="2" t="n"/>
-      <c r="L38" s="2" t="n"/>
-      <c r="M38" s="2" t="n"/>
-      <c r="N38" s="2" t="n"/>
-      <c r="O38" s="2" t="n"/>
-      <c r="P38" s="2" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="12" t="inlineStr">
+      <c r="A38" s="30" t="n"/>
+      <c r="B38" s="31" t="n"/>
+      <c r="C38" s="31" t="n"/>
+      <c r="D38" s="31" t="n"/>
+      <c r="E38" s="32" t="n"/>
+      <c r="F38" s="30" t="n"/>
+      <c r="G38" s="31" t="n"/>
+      <c r="H38" s="31" t="n"/>
+      <c r="I38" s="31" t="n"/>
+      <c r="J38" s="32" t="n"/>
+      <c r="K38" s="30" t="n"/>
+      <c r="L38" s="31" t="n"/>
+      <c r="M38" s="31" t="n"/>
+      <c r="N38" s="31" t="n"/>
+      <c r="O38" s="31" t="n"/>
+      <c r="P38" s="32" t="n"/>
+    </row>
+    <row r="39" ht="32" customHeight="1">
+      <c r="A39" s="23" t="inlineStr">
         <is>
           <t>Rejected or non-conforming goods open a Non-conforming Material Notice and a DÖF (CAPA); Goods Receiving Records are retained 3 years. | البضائع المرفوضة تفتح إشعار عدم مطابقة وإجراءً تصحيحياً.</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="n"/>
-      <c r="G39" s="2" t="n"/>
-      <c r="H39" s="2" t="n"/>
-      <c r="I39" s="2" t="n"/>
-      <c r="J39" s="2" t="n"/>
-      <c r="K39" s="2" t="n"/>
-      <c r="L39" s="2" t="n"/>
-      <c r="M39" s="2" t="n"/>
-      <c r="N39" s="2" t="n"/>
-      <c r="O39" s="2" t="n"/>
-      <c r="P39" s="2" t="n"/>
+      <c r="B39" s="35" t="n"/>
+      <c r="C39" s="35" t="n"/>
+      <c r="D39" s="35" t="n"/>
+      <c r="E39" s="35" t="n"/>
+      <c r="F39" s="35" t="n"/>
+      <c r="G39" s="35" t="n"/>
+      <c r="H39" s="35" t="n"/>
+      <c r="I39" s="35" t="n"/>
+      <c r="J39" s="35" t="n"/>
+      <c r="K39" s="35" t="n"/>
+      <c r="L39" s="35" t="n"/>
+      <c r="M39" s="35" t="n"/>
+      <c r="N39" s="35" t="n"/>
+      <c r="O39" s="35" t="n"/>
+      <c r="P39" s="36" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="176">
+  <mergeCells count="175">
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="P3"/>
     <mergeCell ref="N17:P17"/>
@@ -1396,6 +1618,7 @@
     <mergeCell ref="K11"/>
     <mergeCell ref="J15"/>
     <mergeCell ref="H21"/>
+    <mergeCell ref="D1:K4"/>
     <mergeCell ref="L15"/>
     <mergeCell ref="G19"/>
     <mergeCell ref="I22"/>
@@ -1447,7 +1670,6 @@
     <mergeCell ref="M7:P7"/>
     <mergeCell ref="N22:P22"/>
     <mergeCell ref="B21:D21"/>
-    <mergeCell ref="C1:M4"/>
     <mergeCell ref="N12:P12"/>
     <mergeCell ref="E18:F18"/>
     <mergeCell ref="N4:O4"/>
@@ -1490,7 +1712,6 @@
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="J20"/>
     <mergeCell ref="M16"/>
-    <mergeCell ref="A1:B4"/>
     <mergeCell ref="L20"/>
     <mergeCell ref="K36:P38"/>
     <mergeCell ref="B12:D12"/>

</xml_diff>

<commit_message>
Ortak formların tasarımı geri alındı (organik bölüm ayrı kalır)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6foNXTwf1dGzDjULYpfrk
</commit_message>
<xml_diff>
--- a/formlar/10. Depo ve Sevkiyat/EMS.DP.FRM.08.01. Mal Kabul Kayıt Formu.xlsx
+++ b/formlar/10. Depo ve Sevkiyat/EMS.DP.FRM.08.01. Mal Kabul Kayıt Formu.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Form" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,37 +69,8 @@
       <color rgb="00000000"/>
       <sz val="8"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="28"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -121,18 +92,8 @@
         <fgColor rgb="00F6F7F9"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00006600"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EBF1DE"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="16">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -154,121 +115,11 @@
         <color rgb="009AA3B2"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="009AA3B2"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="009AA3B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="009AA3B2"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="009AA3B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="009AA3B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="009AA3B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="009AA3B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="009AA3B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="009AA3B2"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="009AA3B2"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="009AA3B2"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="009AA3B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="009AA3B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="009AA3B2"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="009AA3B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium"/>
-      <top style="medium"/>
-    </border>
-    <border>
-      <top style="medium"/>
-    </border>
-    <border>
-      <left style="medium"/>
-    </border>
-    <border/>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -302,48 +153,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -421,67 +230,32 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
     <from>
       <col>0</col>
-      <colOff>238124</colOff>
+      <colOff>0</colOff>
       <row>0</row>
-      <rowOff>198193</rowOff>
+      <rowOff>0</rowOff>
     </from>
-    <to>
-      <col>2</col>
-      <colOff>171449</colOff>
-      <row>3</row>
-      <rowOff>205802</rowOff>
-    </to>
+    <ext cx="971550" cy="762000"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>11</col>
-      <colOff>66676</colOff>
-      <row>0</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <to>
-      <col>12</col>
-      <colOff>609600</colOff>
-      <row>3</row>
-      <rowOff>283176</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -796,317 +570,315 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="13" t="n"/>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="15" t="n"/>
-      <c r="D1" s="16" t="inlineStr">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>GOODS RECEIVING RECORD
 سجل استلام البضائع</t>
         </is>
       </c>
-      <c r="E1" s="14" t="n"/>
-      <c r="F1" s="14" t="n"/>
-      <c r="G1" s="14" t="n"/>
-      <c r="H1" s="14" t="n"/>
-      <c r="I1" s="14" t="n"/>
-      <c r="J1" s="14" t="n"/>
-      <c r="K1" s="14" t="n"/>
-      <c r="L1" s="14" t="n"/>
-      <c r="M1" s="14" t="n"/>
-      <c r="N1" s="17" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="2" t="n"/>
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>DATE / التاريخ</t>
         </is>
       </c>
-      <c r="O1" s="18" t="n"/>
-      <c r="P1" s="19" t="inlineStr">
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>….../….../.…</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="20" t="n"/>
-      <c r="B2" s="21" t="n"/>
-      <c r="C2" s="21" t="n"/>
-      <c r="D2" s="21" t="n"/>
-      <c r="E2" s="21" t="n"/>
-      <c r="F2" s="21" t="n"/>
-      <c r="G2" s="21" t="n"/>
-      <c r="H2" s="21" t="n"/>
-      <c r="I2" s="21" t="n"/>
-      <c r="J2" s="21" t="n"/>
-      <c r="K2" s="21" t="n"/>
-      <c r="L2" s="21" t="n"/>
-      <c r="M2" s="21" t="n"/>
-      <c r="N2" s="17" t="inlineStr">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>FORM NUMBER / رقم النموذج</t>
         </is>
       </c>
-      <c r="O2" s="18" t="n"/>
-      <c r="P2" s="22" t="inlineStr">
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="5" t="inlineStr">
         <is>
           <t>EMS.DP.FRM.08.01</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="20" t="n"/>
-      <c r="B3" s="21" t="n"/>
-      <c r="C3" s="21" t="n"/>
-      <c r="D3" s="21" t="n"/>
-      <c r="E3" s="21" t="n"/>
-      <c r="F3" s="21" t="n"/>
-      <c r="G3" s="21" t="n"/>
-      <c r="H3" s="21" t="n"/>
-      <c r="I3" s="21" t="n"/>
-      <c r="J3" s="21" t="n"/>
-      <c r="K3" s="21" t="n"/>
-      <c r="L3" s="21" t="n"/>
-      <c r="M3" s="21" t="n"/>
-      <c r="N3" s="17" t="inlineStr">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>REVISION / المراجعة</t>
         </is>
       </c>
-      <c r="O3" s="18" t="n"/>
-      <c r="P3" s="19" t="inlineStr">
+      <c r="O3" s="2" t="n"/>
+      <c r="P3" s="1" t="inlineStr">
         <is>
           <t>R00</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="20" t="n"/>
-      <c r="B4" s="21" t="n"/>
-      <c r="C4" s="21" t="n"/>
-      <c r="D4" s="21" t="n"/>
-      <c r="E4" s="21" t="n"/>
-      <c r="F4" s="21" t="n"/>
-      <c r="G4" s="21" t="n"/>
-      <c r="H4" s="21" t="n"/>
-      <c r="I4" s="21" t="n"/>
-      <c r="J4" s="21" t="n"/>
-      <c r="K4" s="21" t="n"/>
-      <c r="L4" s="21" t="n"/>
-      <c r="M4" s="21" t="n"/>
-      <c r="N4" s="17" t="inlineStr">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="n"/>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>PUBLIC. DATE / تاريخ النشر</t>
         </is>
       </c>
-      <c r="O4" s="18" t="n"/>
-      <c r="P4" s="19" t="inlineStr">
+      <c r="O4" s="2" t="n"/>
+      <c r="P4" s="1" t="inlineStr">
         <is>
           <t>14.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>RECEIVING INFORMATION / معلومات الاستلام</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n"/>
-      <c r="C6" s="24" t="n"/>
-      <c r="D6" s="24" t="n"/>
-      <c r="E6" s="24" t="n"/>
-      <c r="F6" s="24" t="n"/>
-      <c r="G6" s="24" t="n"/>
-      <c r="H6" s="24" t="n"/>
-      <c r="I6" s="24" t="n"/>
-      <c r="J6" s="24" t="n"/>
-      <c r="K6" s="24" t="n"/>
-      <c r="L6" s="24" t="n"/>
-      <c r="M6" s="24" t="n"/>
-      <c r="N6" s="24" t="n"/>
-      <c r="O6" s="24" t="n"/>
-      <c r="P6" s="25" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n"/>
+      <c r="M6" s="2" t="n"/>
+      <c r="N6" s="2" t="n"/>
+      <c r="O6" s="2" t="n"/>
+      <c r="P6" s="2" t="n"/>
     </row>
     <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Date / Time
 التاريخ / الوقت</t>
         </is>
       </c>
-      <c r="B7" s="24" t="n"/>
-      <c r="C7" s="24" t="n"/>
-      <c r="D7" s="25" t="n"/>
-      <c r="E7" s="26" t="inlineStr">
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Supplier
 المورد</t>
         </is>
       </c>
-      <c r="F7" s="24" t="n"/>
-      <c r="G7" s="24" t="n"/>
-      <c r="H7" s="25" t="n"/>
-      <c r="I7" s="26" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="8" t="n"/>
+      <c r="H7" s="8" t="n"/>
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>Delivery Note No
 رقم إشعار التسليم</t>
         </is>
       </c>
-      <c r="J7" s="24" t="n"/>
-      <c r="K7" s="24" t="n"/>
-      <c r="L7" s="25" t="n"/>
-      <c r="M7" s="26" t="inlineStr">
+      <c r="J7" s="8" t="n"/>
+      <c r="K7" s="8" t="n"/>
+      <c r="L7" s="8" t="n"/>
+      <c r="M7" s="7" t="inlineStr">
         <is>
           <t>Purchase Order No
 رقم أمر الشراء</t>
         </is>
       </c>
-      <c r="N7" s="24" t="n"/>
-      <c r="O7" s="24" t="n"/>
-      <c r="P7" s="25" t="n"/>
+      <c r="N7" s="8" t="n"/>
+      <c r="O7" s="8" t="n"/>
+      <c r="P7" s="8" t="n"/>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Vehicle Plate / Driver
 لوحة المركبة / السائق</t>
         </is>
       </c>
-      <c r="B8" s="24" t="n"/>
-      <c r="C8" s="24" t="n"/>
-      <c r="D8" s="25" t="n"/>
-      <c r="E8" s="26" t="inlineStr">
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Material Type
 نوع المادة (yarn / fabric / chemical / accessory / packaging)</t>
         </is>
       </c>
-      <c r="F8" s="24" t="n"/>
-      <c r="G8" s="24" t="n"/>
-      <c r="H8" s="25" t="n"/>
-      <c r="I8" s="26" t="inlineStr">
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="8" t="n"/>
+      <c r="H8" s="8" t="n"/>
+      <c r="I8" s="7" t="inlineStr">
         <is>
           <t>Warehouse Location
 موقع المستودع</t>
         </is>
       </c>
-      <c r="J8" s="24" t="n"/>
-      <c r="K8" s="24" t="n"/>
-      <c r="L8" s="25" t="n"/>
-      <c r="M8" s="26" t="inlineStr">
+      <c r="J8" s="8" t="n"/>
+      <c r="K8" s="8" t="n"/>
+      <c r="L8" s="8" t="n"/>
+      <c r="M8" s="7" t="inlineStr">
         <is>
           <t>Received By
 المستلم</t>
         </is>
       </c>
-      <c r="N8" s="24" t="n"/>
-      <c r="O8" s="24" t="n"/>
-      <c r="P8" s="25" t="n"/>
-    </row>
-    <row r="9"/>
+      <c r="N8" s="8" t="n"/>
+      <c r="O8" s="8" t="n"/>
+      <c r="P8" s="8" t="n"/>
+    </row>
     <row r="10">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>RECEIVED ITEMS / البنود المستلمة</t>
         </is>
       </c>
-      <c r="B10" s="24" t="n"/>
-      <c r="C10" s="24" t="n"/>
-      <c r="D10" s="24" t="n"/>
-      <c r="E10" s="24" t="n"/>
-      <c r="F10" s="24" t="n"/>
-      <c r="G10" s="24" t="n"/>
-      <c r="H10" s="24" t="n"/>
-      <c r="I10" s="24" t="n"/>
-      <c r="J10" s="24" t="n"/>
-      <c r="K10" s="24" t="n"/>
-      <c r="L10" s="24" t="n"/>
-      <c r="M10" s="24" t="n"/>
-      <c r="N10" s="24" t="n"/>
-      <c r="O10" s="24" t="n"/>
-      <c r="P10" s="25" t="n"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="2" t="n"/>
+      <c r="M10" s="2" t="n"/>
+      <c r="N10" s="2" t="n"/>
+      <c r="O10" s="2" t="n"/>
+      <c r="P10" s="2" t="n"/>
     </row>
     <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B11" s="27" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Item / Description
 الصنف / الوصف</t>
         </is>
       </c>
-      <c r="C11" s="24" t="n"/>
-      <c r="D11" s="25" t="n"/>
-      <c r="E11" s="27" t="inlineStr">
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>Lot / Batch No
 رقم الدفعة</t>
         </is>
       </c>
-      <c r="F11" s="25" t="n"/>
-      <c r="G11" s="27" t="inlineStr">
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>Ordered Qty
 المطلوب</t>
         </is>
       </c>
-      <c r="H11" s="27" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>Delivery Note Qty
 حسب الإشعار</t>
         </is>
       </c>
-      <c r="I11" s="27" t="inlineStr">
+      <c r="I11" s="9" t="inlineStr">
         <is>
           <t>Received Qty
 المستلم</t>
         </is>
       </c>
-      <c r="J11" s="27" t="inlineStr">
+      <c r="J11" s="9" t="inlineStr">
         <is>
           <t>Unit
 الوحدة</t>
         </is>
       </c>
-      <c r="K11" s="27" t="inlineStr">
+      <c r="K11" s="9" t="inlineStr">
         <is>
           <t>Packaging OK
 التغليف سليم</t>
         </is>
       </c>
-      <c r="L11" s="27" t="inlineStr">
+      <c r="L11" s="9" t="inlineStr">
         <is>
           <t>Label OK
 الملصق سليم</t>
         </is>
       </c>
-      <c r="M11" s="27" t="inlineStr">
+      <c r="M11" s="9" t="inlineStr">
         <is>
           <t>Result
 النتيجة (A/R/H)</t>
         </is>
       </c>
-      <c r="N11" s="27" t="inlineStr">
+      <c r="N11" s="9" t="inlineStr">
         <is>
           <t>Remarks
 ملاحظات</t>
         </is>
       </c>
-      <c r="O11" s="24" t="n"/>
-      <c r="P11" s="25" t="n"/>
+      <c r="O11" s="2" t="n"/>
+      <c r="P11" s="2" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="10" t="n">
         <v>1</v>
       </c>
       <c r="B12" s="10" t="n"/>
-      <c r="C12" s="24" t="n"/>
-      <c r="D12" s="25" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
       <c r="E12" s="10" t="n"/>
-      <c r="F12" s="25" t="n"/>
+      <c r="F12" s="2" t="n"/>
       <c r="G12" s="10" t="n"/>
       <c r="H12" s="10" t="n"/>
       <c r="I12" s="10" t="n"/>
@@ -1115,18 +887,18 @@
       <c r="L12" s="10" t="n"/>
       <c r="M12" s="10" t="n"/>
       <c r="N12" s="10" t="n"/>
-      <c r="O12" s="24" t="n"/>
-      <c r="P12" s="25" t="n"/>
+      <c r="O12" s="2" t="n"/>
+      <c r="P12" s="2" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="10" t="n">
         <v>2</v>
       </c>
       <c r="B13" s="10" t="n"/>
-      <c r="C13" s="24" t="n"/>
-      <c r="D13" s="25" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
       <c r="E13" s="10" t="n"/>
-      <c r="F13" s="25" t="n"/>
+      <c r="F13" s="2" t="n"/>
       <c r="G13" s="10" t="n"/>
       <c r="H13" s="10" t="n"/>
       <c r="I13" s="10" t="n"/>
@@ -1135,18 +907,18 @@
       <c r="L13" s="10" t="n"/>
       <c r="M13" s="10" t="n"/>
       <c r="N13" s="10" t="n"/>
-      <c r="O13" s="24" t="n"/>
-      <c r="P13" s="25" t="n"/>
+      <c r="O13" s="2" t="n"/>
+      <c r="P13" s="2" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="10" t="n">
         <v>3</v>
       </c>
       <c r="B14" s="10" t="n"/>
-      <c r="C14" s="24" t="n"/>
-      <c r="D14" s="25" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
       <c r="E14" s="10" t="n"/>
-      <c r="F14" s="25" t="n"/>
+      <c r="F14" s="2" t="n"/>
       <c r="G14" s="10" t="n"/>
       <c r="H14" s="10" t="n"/>
       <c r="I14" s="10" t="n"/>
@@ -1155,18 +927,18 @@
       <c r="L14" s="10" t="n"/>
       <c r="M14" s="10" t="n"/>
       <c r="N14" s="10" t="n"/>
-      <c r="O14" s="24" t="n"/>
-      <c r="P14" s="25" t="n"/>
+      <c r="O14" s="2" t="n"/>
+      <c r="P14" s="2" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="10" t="n">
         <v>4</v>
       </c>
       <c r="B15" s="10" t="n"/>
-      <c r="C15" s="24" t="n"/>
-      <c r="D15" s="25" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
       <c r="E15" s="10" t="n"/>
-      <c r="F15" s="25" t="n"/>
+      <c r="F15" s="2" t="n"/>
       <c r="G15" s="10" t="n"/>
       <c r="H15" s="10" t="n"/>
       <c r="I15" s="10" t="n"/>
@@ -1175,18 +947,18 @@
       <c r="L15" s="10" t="n"/>
       <c r="M15" s="10" t="n"/>
       <c r="N15" s="10" t="n"/>
-      <c r="O15" s="24" t="n"/>
-      <c r="P15" s="25" t="n"/>
+      <c r="O15" s="2" t="n"/>
+      <c r="P15" s="2" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="10" t="n">
         <v>5</v>
       </c>
       <c r="B16" s="10" t="n"/>
-      <c r="C16" s="24" t="n"/>
-      <c r="D16" s="25" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
       <c r="E16" s="10" t="n"/>
-      <c r="F16" s="25" t="n"/>
+      <c r="F16" s="2" t="n"/>
       <c r="G16" s="10" t="n"/>
       <c r="H16" s="10" t="n"/>
       <c r="I16" s="10" t="n"/>
@@ -1195,18 +967,18 @@
       <c r="L16" s="10" t="n"/>
       <c r="M16" s="10" t="n"/>
       <c r="N16" s="10" t="n"/>
-      <c r="O16" s="24" t="n"/>
-      <c r="P16" s="25" t="n"/>
+      <c r="O16" s="2" t="n"/>
+      <c r="P16" s="2" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="10" t="n">
         <v>6</v>
       </c>
       <c r="B17" s="10" t="n"/>
-      <c r="C17" s="24" t="n"/>
-      <c r="D17" s="25" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
       <c r="E17" s="10" t="n"/>
-      <c r="F17" s="25" t="n"/>
+      <c r="F17" s="2" t="n"/>
       <c r="G17" s="10" t="n"/>
       <c r="H17" s="10" t="n"/>
       <c r="I17" s="10" t="n"/>
@@ -1215,18 +987,18 @@
       <c r="L17" s="10" t="n"/>
       <c r="M17" s="10" t="n"/>
       <c r="N17" s="10" t="n"/>
-      <c r="O17" s="24" t="n"/>
-      <c r="P17" s="25" t="n"/>
+      <c r="O17" s="2" t="n"/>
+      <c r="P17" s="2" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="10" t="n">
         <v>7</v>
       </c>
       <c r="B18" s="10" t="n"/>
-      <c r="C18" s="24" t="n"/>
-      <c r="D18" s="25" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
       <c r="E18" s="10" t="n"/>
-      <c r="F18" s="25" t="n"/>
+      <c r="F18" s="2" t="n"/>
       <c r="G18" s="10" t="n"/>
       <c r="H18" s="10" t="n"/>
       <c r="I18" s="10" t="n"/>
@@ -1235,18 +1007,18 @@
       <c r="L18" s="10" t="n"/>
       <c r="M18" s="10" t="n"/>
       <c r="N18" s="10" t="n"/>
-      <c r="O18" s="24" t="n"/>
-      <c r="P18" s="25" t="n"/>
+      <c r="O18" s="2" t="n"/>
+      <c r="P18" s="2" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="10" t="n">
         <v>8</v>
       </c>
       <c r="B19" s="10" t="n"/>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="25" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
       <c r="E19" s="10" t="n"/>
-      <c r="F19" s="25" t="n"/>
+      <c r="F19" s="2" t="n"/>
       <c r="G19" s="10" t="n"/>
       <c r="H19" s="10" t="n"/>
       <c r="I19" s="10" t="n"/>
@@ -1255,18 +1027,18 @@
       <c r="L19" s="10" t="n"/>
       <c r="M19" s="10" t="n"/>
       <c r="N19" s="10" t="n"/>
-      <c r="O19" s="24" t="n"/>
-      <c r="P19" s="25" t="n"/>
+      <c r="O19" s="2" t="n"/>
+      <c r="P19" s="2" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="10" t="n">
         <v>9</v>
       </c>
       <c r="B20" s="10" t="n"/>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="25" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
       <c r="E20" s="10" t="n"/>
-      <c r="F20" s="25" t="n"/>
+      <c r="F20" s="2" t="n"/>
       <c r="G20" s="10" t="n"/>
       <c r="H20" s="10" t="n"/>
       <c r="I20" s="10" t="n"/>
@@ -1275,18 +1047,18 @@
       <c r="L20" s="10" t="n"/>
       <c r="M20" s="10" t="n"/>
       <c r="N20" s="10" t="n"/>
-      <c r="O20" s="24" t="n"/>
-      <c r="P20" s="25" t="n"/>
+      <c r="O20" s="2" t="n"/>
+      <c r="P20" s="2" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="10" t="n">
         <v>10</v>
       </c>
       <c r="B21" s="10" t="n"/>
-      <c r="C21" s="24" t="n"/>
-      <c r="D21" s="25" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
       <c r="E21" s="10" t="n"/>
-      <c r="F21" s="25" t="n"/>
+      <c r="F21" s="2" t="n"/>
       <c r="G21" s="10" t="n"/>
       <c r="H21" s="10" t="n"/>
       <c r="I21" s="10" t="n"/>
@@ -1295,18 +1067,18 @@
       <c r="L21" s="10" t="n"/>
       <c r="M21" s="10" t="n"/>
       <c r="N21" s="10" t="n"/>
-      <c r="O21" s="24" t="n"/>
-      <c r="P21" s="25" t="n"/>
+      <c r="O21" s="2" t="n"/>
+      <c r="P21" s="2" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="10" t="n">
         <v>11</v>
       </c>
       <c r="B22" s="10" t="n"/>
-      <c r="C22" s="24" t="n"/>
-      <c r="D22" s="25" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
       <c r="E22" s="10" t="n"/>
-      <c r="F22" s="25" t="n"/>
+      <c r="F22" s="2" t="n"/>
       <c r="G22" s="10" t="n"/>
       <c r="H22" s="10" t="n"/>
       <c r="I22" s="10" t="n"/>
@@ -1315,18 +1087,18 @@
       <c r="L22" s="10" t="n"/>
       <c r="M22" s="10" t="n"/>
       <c r="N22" s="10" t="n"/>
-      <c r="O22" s="24" t="n"/>
-      <c r="P22" s="25" t="n"/>
+      <c r="O22" s="2" t="n"/>
+      <c r="P22" s="2" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="10" t="n">
         <v>12</v>
       </c>
       <c r="B23" s="10" t="n"/>
-      <c r="C23" s="24" t="n"/>
-      <c r="D23" s="25" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
       <c r="E23" s="10" t="n"/>
-      <c r="F23" s="25" t="n"/>
+      <c r="F23" s="2" t="n"/>
       <c r="G23" s="10" t="n"/>
       <c r="H23" s="10" t="n"/>
       <c r="I23" s="10" t="n"/>
@@ -1335,31 +1107,30 @@
       <c r="L23" s="10" t="n"/>
       <c r="M23" s="10" t="n"/>
       <c r="N23" s="10" t="n"/>
-      <c r="O23" s="24" t="n"/>
-      <c r="P23" s="25" t="n"/>
-    </row>
-    <row r="24"/>
+      <c r="O23" s="2" t="n"/>
+      <c r="P23" s="2" t="n"/>
+    </row>
     <row r="25">
-      <c r="A25" s="23" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>CHECKS / الفحوصات</t>
         </is>
       </c>
-      <c r="B25" s="24" t="n"/>
-      <c r="C25" s="24" t="n"/>
-      <c r="D25" s="24" t="n"/>
-      <c r="E25" s="24" t="n"/>
-      <c r="F25" s="24" t="n"/>
-      <c r="G25" s="24" t="n"/>
-      <c r="H25" s="24" t="n"/>
-      <c r="I25" s="24" t="n"/>
-      <c r="J25" s="24" t="n"/>
-      <c r="K25" s="24" t="n"/>
-      <c r="L25" s="24" t="n"/>
-      <c r="M25" s="24" t="n"/>
-      <c r="N25" s="24" t="n"/>
-      <c r="O25" s="24" t="n"/>
-      <c r="P25" s="25" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" s="2" t="n"/>
+      <c r="K25" s="2" t="n"/>
+      <c r="L25" s="2" t="n"/>
+      <c r="M25" s="2" t="n"/>
+      <c r="N25" s="2" t="n"/>
+      <c r="O25" s="2" t="n"/>
+      <c r="P25" s="2" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
@@ -1367,44 +1138,43 @@
           <t>☐ Delivery note matches order / الإشعار مطابق للطلب   ☐ Quantity and lot match / الكمية والدفعة مطابقة   ☐ Packaging undamaged / التغليف غير تالف   ☐ Labels readable / الملصقات واضحة   ☐ Certificates and MSDS received / الشهادات ونشرة السلامة   ☐ Sent to quality inspection / أرسل لفحص الجودة</t>
         </is>
       </c>
-      <c r="B26" s="24" t="n"/>
-      <c r="C26" s="24" t="n"/>
-      <c r="D26" s="24" t="n"/>
-      <c r="E26" s="24" t="n"/>
-      <c r="F26" s="24" t="n"/>
-      <c r="G26" s="24" t="n"/>
-      <c r="H26" s="24" t="n"/>
-      <c r="I26" s="24" t="n"/>
-      <c r="J26" s="24" t="n"/>
-      <c r="K26" s="24" t="n"/>
-      <c r="L26" s="24" t="n"/>
-      <c r="M26" s="24" t="n"/>
-      <c r="N26" s="24" t="n"/>
-      <c r="O26" s="24" t="n"/>
-      <c r="P26" s="25" t="n"/>
-    </row>
-    <row r="27"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="2" t="n"/>
+      <c r="J26" s="2" t="n"/>
+      <c r="K26" s="2" t="n"/>
+      <c r="L26" s="2" t="n"/>
+      <c r="M26" s="2" t="n"/>
+      <c r="N26" s="2" t="n"/>
+      <c r="O26" s="2" t="n"/>
+      <c r="P26" s="2" t="n"/>
+    </row>
     <row r="28">
-      <c r="A28" s="23" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>DECISION / القرار</t>
         </is>
       </c>
-      <c r="B28" s="24" t="n"/>
-      <c r="C28" s="24" t="n"/>
-      <c r="D28" s="24" t="n"/>
-      <c r="E28" s="24" t="n"/>
-      <c r="F28" s="24" t="n"/>
-      <c r="G28" s="24" t="n"/>
-      <c r="H28" s="24" t="n"/>
-      <c r="I28" s="24" t="n"/>
-      <c r="J28" s="24" t="n"/>
-      <c r="K28" s="24" t="n"/>
-      <c r="L28" s="24" t="n"/>
-      <c r="M28" s="24" t="n"/>
-      <c r="N28" s="24" t="n"/>
-      <c r="O28" s="24" t="n"/>
-      <c r="P28" s="25" t="n"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="2" t="n"/>
+      <c r="J28" s="2" t="n"/>
+      <c r="K28" s="2" t="n"/>
+      <c r="L28" s="2" t="n"/>
+      <c r="M28" s="2" t="n"/>
+      <c r="N28" s="2" t="n"/>
+      <c r="O28" s="2" t="n"/>
+      <c r="P28" s="2" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
@@ -1412,44 +1182,43 @@
           <t>☐ Accepted - stored / مقبول - مخزن   ☐ Hold - awaiting inspection / معلق بانتظار الفحص   ☐ Rejected - Non-conforming Material Notice / مرفوض</t>
         </is>
       </c>
-      <c r="B29" s="24" t="n"/>
-      <c r="C29" s="24" t="n"/>
-      <c r="D29" s="24" t="n"/>
-      <c r="E29" s="24" t="n"/>
-      <c r="F29" s="24" t="n"/>
-      <c r="G29" s="24" t="n"/>
-      <c r="H29" s="24" t="n"/>
-      <c r="I29" s="24" t="n"/>
-      <c r="J29" s="24" t="n"/>
-      <c r="K29" s="24" t="n"/>
-      <c r="L29" s="24" t="n"/>
-      <c r="M29" s="24" t="n"/>
-      <c r="N29" s="24" t="n"/>
-      <c r="O29" s="24" t="n"/>
-      <c r="P29" s="25" t="n"/>
-    </row>
-    <row r="30"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
+      <c r="I29" s="2" t="n"/>
+      <c r="J29" s="2" t="n"/>
+      <c r="K29" s="2" t="n"/>
+      <c r="L29" s="2" t="n"/>
+      <c r="M29" s="2" t="n"/>
+      <c r="N29" s="2" t="n"/>
+      <c r="O29" s="2" t="n"/>
+      <c r="P29" s="2" t="n"/>
+    </row>
     <row r="31">
-      <c r="A31" s="23" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>NOTES / ملاحظات</t>
         </is>
       </c>
-      <c r="B31" s="24" t="n"/>
-      <c r="C31" s="24" t="n"/>
-      <c r="D31" s="24" t="n"/>
-      <c r="E31" s="24" t="n"/>
-      <c r="F31" s="24" t="n"/>
-      <c r="G31" s="24" t="n"/>
-      <c r="H31" s="24" t="n"/>
-      <c r="I31" s="24" t="n"/>
-      <c r="J31" s="24" t="n"/>
-      <c r="K31" s="24" t="n"/>
-      <c r="L31" s="24" t="n"/>
-      <c r="M31" s="24" t="n"/>
-      <c r="N31" s="24" t="n"/>
-      <c r="O31" s="24" t="n"/>
-      <c r="P31" s="25" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" s="2" t="n"/>
+      <c r="K31" s="2" t="n"/>
+      <c r="L31" s="2" t="n"/>
+      <c r="M31" s="2" t="n"/>
+      <c r="N31" s="2" t="n"/>
+      <c r="O31" s="2" t="n"/>
+      <c r="P31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
@@ -1457,139 +1226,148 @@
           <t>Shortages, damage, discrepancies and photo references.</t>
         </is>
       </c>
-      <c r="B32" s="28" t="n"/>
-      <c r="C32" s="28" t="n"/>
-      <c r="D32" s="28" t="n"/>
-      <c r="E32" s="28" t="n"/>
-      <c r="F32" s="28" t="n"/>
-      <c r="G32" s="28" t="n"/>
-      <c r="H32" s="28" t="n"/>
-      <c r="I32" s="28" t="n"/>
-      <c r="J32" s="28" t="n"/>
-      <c r="K32" s="28" t="n"/>
-      <c r="L32" s="28" t="n"/>
-      <c r="M32" s="28" t="n"/>
-      <c r="N32" s="28" t="n"/>
-      <c r="O32" s="28" t="n"/>
-      <c r="P32" s="29" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="2" t="n"/>
+      <c r="K32" s="2" t="n"/>
+      <c r="L32" s="2" t="n"/>
+      <c r="M32" s="2" t="n"/>
+      <c r="N32" s="2" t="n"/>
+      <c r="O32" s="2" t="n"/>
+      <c r="P32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="30" t="n"/>
-      <c r="B33" s="31" t="n"/>
-      <c r="C33" s="31" t="n"/>
-      <c r="D33" s="31" t="n"/>
-      <c r="E33" s="31" t="n"/>
-      <c r="F33" s="31" t="n"/>
-      <c r="G33" s="31" t="n"/>
-      <c r="H33" s="31" t="n"/>
-      <c r="I33" s="31" t="n"/>
-      <c r="J33" s="31" t="n"/>
-      <c r="K33" s="31" t="n"/>
-      <c r="L33" s="31" t="n"/>
-      <c r="M33" s="31" t="n"/>
-      <c r="N33" s="31" t="n"/>
-      <c r="O33" s="31" t="n"/>
-      <c r="P33" s="32" t="n"/>
-    </row>
-    <row r="34"/>
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="n"/>
+      <c r="K33" s="2" t="n"/>
+      <c r="L33" s="2" t="n"/>
+      <c r="M33" s="2" t="n"/>
+      <c r="N33" s="2" t="n"/>
+      <c r="O33" s="2" t="n"/>
+      <c r="P33" s="2" t="n"/>
+    </row>
     <row r="35">
-      <c r="A35" s="27" t="inlineStr">
+      <c r="A35" s="9" t="inlineStr">
         <is>
           <t>Warehouse / المستودع</t>
         </is>
       </c>
-      <c r="B35" s="24" t="n"/>
-      <c r="C35" s="24" t="n"/>
-      <c r="D35" s="24" t="n"/>
-      <c r="E35" s="25" t="n"/>
-      <c r="F35" s="27" t="inlineStr">
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="9" t="inlineStr">
         <is>
           <t>Quality / الجودة</t>
         </is>
       </c>
-      <c r="G35" s="24" t="n"/>
-      <c r="H35" s="24" t="n"/>
-      <c r="I35" s="24" t="n"/>
-      <c r="J35" s="25" t="n"/>
-      <c r="K35" s="27" t="inlineStr">
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="n"/>
+      <c r="K35" s="9" t="inlineStr">
         <is>
           <t>Purchasing / المشتريات</t>
         </is>
       </c>
-      <c r="L35" s="24" t="n"/>
-      <c r="M35" s="24" t="n"/>
-      <c r="N35" s="24" t="n"/>
-      <c r="O35" s="24" t="n"/>
-      <c r="P35" s="25" t="n"/>
+      <c r="L35" s="2" t="n"/>
+      <c r="M35" s="2" t="n"/>
+      <c r="N35" s="2" t="n"/>
+      <c r="O35" s="2" t="n"/>
+      <c r="P35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n"/>
-      <c r="B36" s="28" t="n"/>
-      <c r="C36" s="28" t="n"/>
-      <c r="D36" s="28" t="n"/>
-      <c r="E36" s="29" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
       <c r="F36" s="1" t="n"/>
-      <c r="G36" s="28" t="n"/>
-      <c r="H36" s="28" t="n"/>
-      <c r="I36" s="28" t="n"/>
-      <c r="J36" s="29" t="n"/>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+      <c r="I36" s="2" t="n"/>
+      <c r="J36" s="2" t="n"/>
       <c r="K36" s="1" t="n"/>
-      <c r="L36" s="28" t="n"/>
-      <c r="M36" s="28" t="n"/>
-      <c r="N36" s="28" t="n"/>
-      <c r="O36" s="28" t="n"/>
-      <c r="P36" s="29" t="n"/>
+      <c r="L36" s="2" t="n"/>
+      <c r="M36" s="2" t="n"/>
+      <c r="N36" s="2" t="n"/>
+      <c r="O36" s="2" t="n"/>
+      <c r="P36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="33" t="n"/>
-      <c r="E37" s="34" t="n"/>
-      <c r="F37" s="33" t="n"/>
-      <c r="J37" s="34" t="n"/>
-      <c r="K37" s="33" t="n"/>
-      <c r="P37" s="34" t="n"/>
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
+      <c r="I37" s="2" t="n"/>
+      <c r="J37" s="2" t="n"/>
+      <c r="K37" s="2" t="n"/>
+      <c r="L37" s="2" t="n"/>
+      <c r="M37" s="2" t="n"/>
+      <c r="N37" s="2" t="n"/>
+      <c r="O37" s="2" t="n"/>
+      <c r="P37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="30" t="n"/>
-      <c r="B38" s="31" t="n"/>
-      <c r="C38" s="31" t="n"/>
-      <c r="D38" s="31" t="n"/>
-      <c r="E38" s="32" t="n"/>
-      <c r="F38" s="30" t="n"/>
-      <c r="G38" s="31" t="n"/>
-      <c r="H38" s="31" t="n"/>
-      <c r="I38" s="31" t="n"/>
-      <c r="J38" s="32" t="n"/>
-      <c r="K38" s="30" t="n"/>
-      <c r="L38" s="31" t="n"/>
-      <c r="M38" s="31" t="n"/>
-      <c r="N38" s="31" t="n"/>
-      <c r="O38" s="31" t="n"/>
-      <c r="P38" s="32" t="n"/>
-    </row>
-    <row r="39" ht="32" customHeight="1">
-      <c r="A39" s="23" t="inlineStr">
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="n"/>
+      <c r="J38" s="2" t="n"/>
+      <c r="K38" s="2" t="n"/>
+      <c r="L38" s="2" t="n"/>
+      <c r="M38" s="2" t="n"/>
+      <c r="N38" s="2" t="n"/>
+      <c r="O38" s="2" t="n"/>
+      <c r="P38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t>Rejected or non-conforming goods open a Non-conforming Material Notice and a DÖF (CAPA); Goods Receiving Records are retained 3 years. | البضائع المرفوضة تفتح إشعار عدم مطابقة وإجراءً تصحيحياً.</t>
         </is>
       </c>
-      <c r="B39" s="35" t="n"/>
-      <c r="C39" s="35" t="n"/>
-      <c r="D39" s="35" t="n"/>
-      <c r="E39" s="35" t="n"/>
-      <c r="F39" s="35" t="n"/>
-      <c r="G39" s="35" t="n"/>
-      <c r="H39" s="35" t="n"/>
-      <c r="I39" s="35" t="n"/>
-      <c r="J39" s="35" t="n"/>
-      <c r="K39" s="35" t="n"/>
-      <c r="L39" s="35" t="n"/>
-      <c r="M39" s="35" t="n"/>
-      <c r="N39" s="35" t="n"/>
-      <c r="O39" s="35" t="n"/>
-      <c r="P39" s="36" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="n"/>
+      <c r="J39" s="2" t="n"/>
+      <c r="K39" s="2" t="n"/>
+      <c r="L39" s="2" t="n"/>
+      <c r="M39" s="2" t="n"/>
+      <c r="N39" s="2" t="n"/>
+      <c r="O39" s="2" t="n"/>
+      <c r="P39" s="2" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="175">
+  <mergeCells count="176">
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="P3"/>
     <mergeCell ref="N17:P17"/>
@@ -1618,7 +1396,6 @@
     <mergeCell ref="K11"/>
     <mergeCell ref="J15"/>
     <mergeCell ref="H21"/>
-    <mergeCell ref="D1:K4"/>
     <mergeCell ref="L15"/>
     <mergeCell ref="G19"/>
     <mergeCell ref="I22"/>
@@ -1670,6 +1447,7 @@
     <mergeCell ref="M7:P7"/>
     <mergeCell ref="N22:P22"/>
     <mergeCell ref="B21:D21"/>
+    <mergeCell ref="C1:M4"/>
     <mergeCell ref="N12:P12"/>
     <mergeCell ref="E18:F18"/>
     <mergeCell ref="N4:O4"/>
@@ -1712,6 +1490,7 @@
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="J20"/>
     <mergeCell ref="M16"/>
+    <mergeCell ref="A1:B4"/>
     <mergeCell ref="L20"/>
     <mergeCell ref="K36:P38"/>
     <mergeCell ref="B12:D12"/>

</xml_diff>